<commit_message>
docs(idts-100): finalize mentor-ready SAP490 pack
</commit_message>
<xml_diff>
--- a/docs/sap490/generated/Functional_Test_IDTS_SAP01_en_v0.2.xlsx
+++ b/docs/sap490/generated/Functional_Test_IDTS_SAP01_en_v0.2.xlsx
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="155">
   <si>
     <t xml:space="preserve">Functional Test</t>
   </si>
@@ -275,15 +275,18 @@
     <t xml:space="preserve">Preconditions: Authenticated Tester; at least one similar and one unrelated bug.
 Data: A new login-failure description and classification context.
 Expected: Relevant candidates are shown as advice; ignoring them does not mutate data or block create.
-Actual / postcondition: Not run | No automatic duplicate relation exists.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pending</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Command: N/A
-Evidence: N/A
-Defects / limit: None | No fresh UI/API duplicate review execution in this remediation.</t>
+Actual / postcondition: Passed on Render Shared QA. The API and Fiori dialog returned review-only duplicate guidance, covered the no-result state, and did not mutate Bug workflow data. | No automatic duplicate relation exists.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IDTS-100 automated acceptance under DonHV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-07-24T20:42:48+07:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Command: node scripts/qa/test-idts100-shared-qa-lifecycle.js and focused browser/API harnesses
+Evidence: docs/pm/evidence/idts-100/shared-qa-ai/render-ai-smoke.json, docs/pm/evidence/idts-100/shared-qa-ai-browser/all-review-actions/shared-qa-ai-browser.json
+Defects / limit: None | Agent-executed acceptance evidence; formal human UAT sign-off is tracked separately.</t>
   </si>
   <si>
     <t xml:space="preserve">FT-CLASS-ASSIGN-001</t>
@@ -297,12 +300,12 @@
     <t xml:space="preserve">Preconditions: Active classification pairs and Developer Responsibilities exist.
 Data: Application Component=Bug Management; Defect Category=Fiori/UI5; one suitable and one unsuitable Developer.
 Expected: Only responsible active candidates are selectable; saved bug is Assigned and ownership persists after reload.
-Actual / postcondition: Not run | Assigned Developer is the technical owner.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Command: N/A
-Evidence: N/A
-Defects / limit: IDTS-56 | Needs fresh browser and persistence evidence.</t>
+Actual / postcondition: Passed on Render Shared QA. Active classification mapping was accepted, an eligible Developer was assigned, direct Developer self-assignment was denied, and the manual Smart Assign review remained available. | Assigned Developer is the technical owner.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Command: node scripts/qa/test-idts100-shared-qa-lifecycle.js and focused browser/API harnesses
+Evidence: docs/pm/evidence/idts-100/shared-qa-lifecycle/shared-qa-lifecycle.json, docs/pm/evidence/idts-100/shared-qa-ai-browser/assignment/idts72-ai-browser-smoke.json
+Defects / limit: IDTS-56 | Agent-executed acceptance evidence; formal human UAT sign-off is tracked separately.</t>
   </si>
   <si>
     <t xml:space="preserve">FT-PENDING-001</t>
@@ -316,12 +319,12 @@
     <t xml:space="preserve">Preconditions: Tester is authenticated and all required bug fields are valid.
 Data: Valid bug with no selected assignee.
 Expected: Bug is Pending Assignment; no Developer is selected automatically; PM/Tester queue owns the next action.
-Actual / postcondition: Not run | Bug awaits explicit assignment.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Command: N/A
-Evidence: N/A
-Defects / limit: None | Needs fresh create/reload evidence.</t>
+Actual / postcondition: Passed on Render Shared QA. Activating a valid draft without an assignee produced PENDING_ASSIGNMENT, no assignee, and PM as the next processing role. | Bug awaits explicit assignment.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Command: node scripts/qa/test-idts100-shared-qa-lifecycle.js and focused browser/API harnesses
+Evidence: docs/pm/evidence/idts-100/shared-qa-lifecycle/shared-qa-lifecycle.json
+Defects / limit: None | Agent-executed acceptance evidence; formal human UAT sign-off is tracked separately.</t>
   </si>
   <si>
     <t xml:space="preserve">FT-REASSIGN-001</t>
@@ -335,12 +338,7 @@
     <t xml:space="preserve">Preconditions: Assigned bug and a second suitable Developer exist.
 Data: Reason: workload balancing.
 Expected: Exactly one assignee remains; history names actor, old/new owner, reason and timestamp.
-Actual / postcondition: Not run | New Developer is technical owner.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Command: N/A
-Evidence: N/A
-Defects / limit: None | PM direct-reassign authorization remains a documented decision dependency; execute with a role allowed by current runtime.</t>
+Actual / postcondition: Passed on Render Shared QA. The bug moved through rejection to Pending Assignment, cleared the assignee, was reassigned, and retained exact history action types. | New Developer is technical owner.</t>
   </si>
   <si>
     <t xml:space="preserve">FT-DEV-INFO-001</t>
@@ -354,12 +352,12 @@
     <t xml:space="preserve">Preconditions: Assigned bug; assigned and non-assigned Developer accounts.
 Data: Reason: missing browser version and exact reproduction step.
 Expected: Wrong role/owner and blank reason are blocked; valid action sets Need More Information and Tester action ownership with audit/notification.
-Actual / postcondition: Not run | Tester must provide information and resubmit.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Command: N/A
-Evidence: N/A
-Defects / limit: None | Needs fresh role matrix and reload evidence.</t>
+Actual / postcondition: Passed on Render Shared QA. The assigned Developer requested more information, a blank reason returned 400, and the Tester resubmitted the bug to the same Developer. | Tester must provide information and resubmit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Command: node scripts/qa/test-idts100-shared-qa-lifecycle.js and focused browser/API harnesses
+Evidence: docs/pm/evidence/idts-100/shared-qa-lifecycle/shared-qa-lifecycle.json, docs/pm/evidence/idts-100/shared-qa-email-brevo-20260724.md
+Defects / limit: None | Agent-executed acceptance evidence; formal human UAT sign-off is tracked separately.</t>
   </si>
   <si>
     <t xml:space="preserve">FT-REJECT-001</t>
@@ -373,12 +371,7 @@
     <t xml:space="preserve">Preconditions: Assigned bug with unsuitable classification or owner.
 Data: Reason: component is Notification, not Dashboard.
 Expected: Blank reason is blocked; valid rejection records follow-up; correction leaves Rejected through Assigned or Pending Assignment, never directly Need More Information.
-Actual / postcondition: Not run | Bug has a clear next technical/queue owner.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Command: N/A
-Evidence: N/A
-Defects / limit: None | Needs full UI/API lifecycle evidence.</t>
+Actual / postcondition: Passed on Render Shared QA. The assigned Developer rejected with a reason; PM returned the bug to the assignment queue and completed correction follow-up by reassigning it. | Bug has a clear next technical/queue owner.</t>
   </si>
   <si>
     <t xml:space="preserve">FT-LIFECYCLE-001</t>
@@ -392,12 +385,7 @@
     <t xml:space="preserve">Preconditions: Bug is In Progress and reproducible.
 Data: Resolution note plus one passing and one failing retest observation.
 Expected: Pass reaches Closed; fail reaches Reopened; required notes, owners and audit remain consistent after reload.
-Actual / postcondition: Not run | Closed has no next processor; Reopened returns to active handling.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Command: N/A
-Evidence: N/A
-Defects / limit: None | No fresh full lifecycle execution in this remediation.</t>
+Actual / postcondition: Passed on Render Shared QA across PM, Tester and Developer sessions: assign, review, progress, information request, resubmit, resolve, retest, close, reopen, reject and reassign all persisted with exact history and notification side effects. | Closed has no next processor; Reopened returns to active handling.</t>
   </si>
   <si>
     <t xml:space="preserve">FT-COMMENT-001</t>
@@ -433,12 +421,12 @@
     <t xml:space="preserve">Preconditions: Authenticated Tester, existing bug and allowed small evidence file.
 Data: Small text/image file, disallowed MIME variant and over-limit boundary file.
 Expected: Allowed evidence persists and downloads; invalid variants are blocked; delete cleans storage and records history.
-Actual / postcondition: Not run | No orphan attachment remains.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Command: npm run qa:comments-attachments:http
-Evidence: scripts/qa/test-comments-attachments.ps1
-Defects / limit: IDTS-55 | The required HTTP command was not run in this remediation; the programmatic comments suite only printed an attachment note.</t>
+Actual / postcondition: Passed on Render Shared QA. Two files selected before save were uploaded after activation, downloaded with matching SHA-256, persisted after redeploy, and one attachment was deleted with the subsequent download returning 404. | No orphan attachment remains.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Command: npm run qa:idts73:browser + supported OData delete verification
+Evidence: docs/pm/evidence/idts-100/shared-qa-attachments/idts73-create-attachments-browser.json, docs/pm/evidence/idts-100/shared-qa-attachments/delete-verification-20260724.md
+Defects / limit: IDTS-55 | Agent-executed acceptance evidence; formal human UAT sign-off is tracked separately.</t>
   </si>
   <si>
     <t xml:space="preserve">FT-NOTIF-001</t>
@@ -496,12 +484,12 @@
     <t xml:space="preserve">Preconditions: Authenticated user; AI disabled and controlled suggestion modes available.
 Data: Similar/classification/handoff suggestion with safe and malformed variants.
 Expected: Suggestion never changes assignment, classification or lifecycle automatically; normal workflow remains usable.
-Actual / postcondition: Not run | Bug remains unchanged unless an authorized user separately applies a normal action.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Command: N/A
-Evidence: N/A
-Defects / limit: IDTS-78 | REG-AI-20260723 proves provider safety only, not this full human-review business flow.</t>
+Actual / postcondition: Passed for disabled-provider acceptance on Render Shared QA. Similar Bugs, Classification, Handoff Summary and Smart Assignment were review-only, safe, browser-visible and did not mutate workflow. Live OpenAI provider remains NOT ACCEPTED by decision. | Bug remains unchanged unless an authorized user separately applies a normal action.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Command: node scripts/qa/test-idts100-shared-qa-lifecycle.js and focused browser/API harnesses
+Evidence: docs/pm/evidence/idts-100/shared-qa-ai/render-ai-smoke.json, docs/pm/evidence/idts-100/shared-qa-ai-browser/all-review-actions/shared-qa-ai-browser.json, docs/pm/evidence/idts-100/shared-qa-ai-browser/assignment/idts72-ai-browser-smoke.json
+Defects / limit: IDTS-78 | Agent-executed acceptance evidence; formal human UAT sign-off is tracked separately.</t>
   </si>
   <si>
     <t xml:space="preserve">Run ID / exact command</t>
@@ -5493,24 +5481,28 @@
       <c r="AU12" s="53"/>
       <c r="AV12" s="53"/>
       <c r="AW12" s="53"/>
-      <c r="AX12" s="54"/>
+      <c r="AX12" s="54" t="s">
+        <v>64</v>
+      </c>
       <c r="AY12" s="54"/>
       <c r="AZ12" s="54"/>
       <c r="BA12" s="54"/>
       <c r="BB12" s="54"/>
       <c r="BC12" s="54"/>
-      <c r="BD12" s="55"/>
+      <c r="BD12" s="55" t="s">
+        <v>65</v>
+      </c>
       <c r="BE12" s="55"/>
       <c r="BF12" s="55"/>
       <c r="BG12" s="55"/>
       <c r="BH12" s="55"/>
       <c r="BI12" s="55"/>
       <c r="BJ12" s="54" t="s">
-        <v>64</v>
+        <v>46</v>
       </c>
       <c r="BK12" s="54"/>
       <c r="BL12" s="56" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="BM12" s="56"/>
       <c r="BN12" s="56"/>
@@ -5526,12 +5518,12 @@
     <row r="13" customFormat="false" ht="180" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="43"/>
       <c r="B13" s="57" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C13" s="57"/>
       <c r="D13" s="57"/>
       <c r="E13" s="53" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F13" s="53"/>
       <c r="G13" s="53"/>
@@ -5553,7 +5545,7 @@
       <c r="W13" s="53"/>
       <c r="X13" s="53"/>
       <c r="Y13" s="53" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Z13" s="53"/>
       <c r="AA13" s="53"/>
@@ -5579,24 +5571,28 @@
       <c r="AU13" s="53"/>
       <c r="AV13" s="53"/>
       <c r="AW13" s="53"/>
-      <c r="AX13" s="54"/>
+      <c r="AX13" s="54" t="s">
+        <v>64</v>
+      </c>
       <c r="AY13" s="54"/>
       <c r="AZ13" s="54"/>
       <c r="BA13" s="54"/>
       <c r="BB13" s="54"/>
       <c r="BC13" s="54"/>
-      <c r="BD13" s="55"/>
+      <c r="BD13" s="55" t="s">
+        <v>65</v>
+      </c>
       <c r="BE13" s="55"/>
       <c r="BF13" s="55"/>
       <c r="BG13" s="55"/>
       <c r="BH13" s="55"/>
       <c r="BI13" s="55"/>
       <c r="BJ13" s="54" t="s">
-        <v>64</v>
+        <v>46</v>
       </c>
       <c r="BK13" s="54"/>
       <c r="BL13" s="56" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="BM13" s="56"/>
       <c r="BN13" s="56"/>
@@ -5612,12 +5608,12 @@
     <row r="14" customFormat="false" ht="180" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="43"/>
       <c r="B14" s="51" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C14" s="51"/>
       <c r="D14" s="51"/>
       <c r="E14" s="52" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F14" s="52"/>
       <c r="G14" s="52"/>
@@ -5639,7 +5635,7 @@
       <c r="W14" s="52"/>
       <c r="X14" s="52"/>
       <c r="Y14" s="52" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="Z14" s="52"/>
       <c r="AA14" s="52"/>
@@ -5665,24 +5661,28 @@
       <c r="AU14" s="52"/>
       <c r="AV14" s="52"/>
       <c r="AW14" s="52"/>
-      <c r="AX14" s="54"/>
+      <c r="AX14" s="54" t="s">
+        <v>64</v>
+      </c>
       <c r="AY14" s="54"/>
       <c r="AZ14" s="54"/>
       <c r="BA14" s="54"/>
       <c r="BB14" s="54"/>
       <c r="BC14" s="54"/>
-      <c r="BD14" s="55"/>
+      <c r="BD14" s="55" t="s">
+        <v>65</v>
+      </c>
       <c r="BE14" s="55"/>
       <c r="BF14" s="55"/>
       <c r="BG14" s="55"/>
       <c r="BH14" s="55"/>
       <c r="BI14" s="55"/>
       <c r="BJ14" s="54" t="s">
-        <v>64</v>
+        <v>46</v>
       </c>
       <c r="BK14" s="54"/>
       <c r="BL14" s="56" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="BM14" s="56"/>
       <c r="BN14" s="56"/>
@@ -5698,12 +5698,12 @@
     <row r="15" customFormat="false" ht="180" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="43"/>
       <c r="B15" s="57" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C15" s="57"/>
       <c r="D15" s="57"/>
       <c r="E15" s="53" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F15" s="53"/>
       <c r="G15" s="53"/>
@@ -5725,7 +5725,7 @@
       <c r="W15" s="53"/>
       <c r="X15" s="53"/>
       <c r="Y15" s="53" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="Z15" s="53"/>
       <c r="AA15" s="53"/>
@@ -5751,24 +5751,28 @@
       <c r="AU15" s="53"/>
       <c r="AV15" s="53"/>
       <c r="AW15" s="53"/>
-      <c r="AX15" s="54"/>
+      <c r="AX15" s="54" t="s">
+        <v>64</v>
+      </c>
       <c r="AY15" s="54"/>
       <c r="AZ15" s="54"/>
       <c r="BA15" s="54"/>
       <c r="BB15" s="54"/>
       <c r="BC15" s="54"/>
-      <c r="BD15" s="55"/>
+      <c r="BD15" s="55" t="s">
+        <v>65</v>
+      </c>
       <c r="BE15" s="55"/>
       <c r="BF15" s="55"/>
       <c r="BG15" s="55"/>
       <c r="BH15" s="55"/>
       <c r="BI15" s="55"/>
       <c r="BJ15" s="54" t="s">
-        <v>64</v>
+        <v>46</v>
       </c>
       <c r="BK15" s="54"/>
       <c r="BL15" s="56" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="BM15" s="56"/>
       <c r="BN15" s="56"/>
@@ -5837,20 +5841,24 @@
       <c r="AU16" s="53"/>
       <c r="AV16" s="53"/>
       <c r="AW16" s="53"/>
-      <c r="AX16" s="54"/>
+      <c r="AX16" s="54" t="s">
+        <v>64</v>
+      </c>
       <c r="AY16" s="54"/>
       <c r="AZ16" s="54"/>
       <c r="BA16" s="54"/>
       <c r="BB16" s="54"/>
       <c r="BC16" s="54"/>
-      <c r="BD16" s="55"/>
+      <c r="BD16" s="55" t="s">
+        <v>65</v>
+      </c>
       <c r="BE16" s="55"/>
       <c r="BF16" s="55"/>
       <c r="BG16" s="55"/>
       <c r="BH16" s="55"/>
       <c r="BI16" s="55"/>
       <c r="BJ16" s="54" t="s">
-        <v>64</v>
+        <v>46</v>
       </c>
       <c r="BK16" s="54"/>
       <c r="BL16" s="56" t="s">
@@ -5923,24 +5931,28 @@
       <c r="AU17" s="53"/>
       <c r="AV17" s="53"/>
       <c r="AW17" s="53"/>
-      <c r="AX17" s="54"/>
+      <c r="AX17" s="54" t="s">
+        <v>64</v>
+      </c>
       <c r="AY17" s="54"/>
       <c r="AZ17" s="54"/>
       <c r="BA17" s="54"/>
       <c r="BB17" s="54"/>
       <c r="BC17" s="54"/>
-      <c r="BD17" s="55"/>
+      <c r="BD17" s="55" t="s">
+        <v>65</v>
+      </c>
       <c r="BE17" s="55"/>
       <c r="BF17" s="55"/>
       <c r="BG17" s="55"/>
       <c r="BH17" s="55"/>
       <c r="BI17" s="55"/>
       <c r="BJ17" s="54" t="s">
-        <v>64</v>
+        <v>46</v>
       </c>
       <c r="BK17" s="54"/>
       <c r="BL17" s="56" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="BM17" s="56"/>
       <c r="BN17" s="56"/>
@@ -5956,12 +5968,12 @@
     <row r="18" customFormat="false" ht="180" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="43"/>
       <c r="B18" s="57" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C18" s="57"/>
       <c r="D18" s="57"/>
       <c r="E18" s="53" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F18" s="53"/>
       <c r="G18" s="53"/>
@@ -5983,7 +5995,7 @@
       <c r="W18" s="53"/>
       <c r="X18" s="53"/>
       <c r="Y18" s="53" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="Z18" s="53"/>
       <c r="AA18" s="53"/>
@@ -6009,24 +6021,28 @@
       <c r="AU18" s="53"/>
       <c r="AV18" s="53"/>
       <c r="AW18" s="53"/>
-      <c r="AX18" s="54"/>
+      <c r="AX18" s="54" t="s">
+        <v>64</v>
+      </c>
       <c r="AY18" s="54"/>
       <c r="AZ18" s="54"/>
       <c r="BA18" s="54"/>
       <c r="BB18" s="54"/>
       <c r="BC18" s="54"/>
-      <c r="BD18" s="55"/>
+      <c r="BD18" s="55" t="s">
+        <v>65</v>
+      </c>
       <c r="BE18" s="55"/>
       <c r="BF18" s="55"/>
       <c r="BG18" s="55"/>
       <c r="BH18" s="55"/>
       <c r="BI18" s="55"/>
       <c r="BJ18" s="54" t="s">
-        <v>64</v>
+        <v>46</v>
       </c>
       <c r="BK18" s="54"/>
       <c r="BL18" s="56" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="BM18" s="56"/>
       <c r="BN18" s="56"/>
@@ -6042,12 +6058,12 @@
     <row r="19" customFormat="false" ht="180" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="43"/>
       <c r="B19" s="51" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C19" s="51"/>
       <c r="D19" s="51"/>
       <c r="E19" s="52" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F19" s="52"/>
       <c r="G19" s="52"/>
@@ -6069,7 +6085,7 @@
       <c r="W19" s="52"/>
       <c r="X19" s="52"/>
       <c r="Y19" s="53" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="Z19" s="53"/>
       <c r="AA19" s="53"/>
@@ -6104,7 +6120,7 @@
       <c r="BB19" s="54"/>
       <c r="BC19" s="54"/>
       <c r="BD19" s="55" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="BE19" s="55"/>
       <c r="BF19" s="55"/>
@@ -6116,7 +6132,7 @@
       </c>
       <c r="BK19" s="54"/>
       <c r="BL19" s="58" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="BM19" s="58"/>
       <c r="BN19" s="58"/>
@@ -6132,12 +6148,12 @@
     <row r="20" customFormat="false" ht="180" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="43"/>
       <c r="B20" s="57" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C20" s="57"/>
       <c r="D20" s="57"/>
       <c r="E20" s="53" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F20" s="53"/>
       <c r="G20" s="53"/>
@@ -6159,7 +6175,7 @@
       <c r="W20" s="53"/>
       <c r="X20" s="53"/>
       <c r="Y20" s="53" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="Z20" s="53"/>
       <c r="AA20" s="53"/>
@@ -6185,24 +6201,28 @@
       <c r="AU20" s="53"/>
       <c r="AV20" s="53"/>
       <c r="AW20" s="53"/>
-      <c r="AX20" s="54"/>
+      <c r="AX20" s="54" t="s">
+        <v>64</v>
+      </c>
       <c r="AY20" s="54"/>
       <c r="AZ20" s="54"/>
       <c r="BA20" s="54"/>
       <c r="BB20" s="54"/>
       <c r="BC20" s="54"/>
-      <c r="BD20" s="55"/>
+      <c r="BD20" s="55" t="s">
+        <v>65</v>
+      </c>
       <c r="BE20" s="55"/>
       <c r="BF20" s="55"/>
       <c r="BG20" s="55"/>
       <c r="BH20" s="55"/>
       <c r="BI20" s="55"/>
       <c r="BJ20" s="54" t="s">
-        <v>64</v>
+        <v>46</v>
       </c>
       <c r="BK20" s="54"/>
       <c r="BL20" s="58" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="BM20" s="58"/>
       <c r="BN20" s="58"/>
@@ -6218,12 +6238,12 @@
     <row r="21" customFormat="false" ht="180" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="43"/>
       <c r="B21" s="57" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C21" s="57"/>
       <c r="D21" s="57"/>
       <c r="E21" s="53" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F21" s="53"/>
       <c r="G21" s="53"/>
@@ -6245,7 +6265,7 @@
       <c r="W21" s="53"/>
       <c r="X21" s="53"/>
       <c r="Y21" s="53" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="Z21" s="53"/>
       <c r="AA21" s="53"/>
@@ -6280,7 +6300,7 @@
       <c r="BB21" s="54"/>
       <c r="BC21" s="54"/>
       <c r="BD21" s="55" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="BE21" s="55"/>
       <c r="BF21" s="55"/>
@@ -6292,7 +6312,7 @@
       </c>
       <c r="BK21" s="54"/>
       <c r="BL21" s="58" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="BM21" s="58"/>
       <c r="BN21" s="58"/>
@@ -6308,12 +6328,12 @@
     <row r="22" customFormat="false" ht="180" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="43"/>
       <c r="B22" s="57" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C22" s="57"/>
       <c r="D22" s="57"/>
       <c r="E22" s="53" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F22" s="53"/>
       <c r="G22" s="53"/>
@@ -6335,7 +6355,7 @@
       <c r="W22" s="53"/>
       <c r="X22" s="53"/>
       <c r="Y22" s="53" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="Z22" s="53"/>
       <c r="AA22" s="53"/>
@@ -6370,7 +6390,7 @@
       <c r="BB22" s="54"/>
       <c r="BC22" s="54"/>
       <c r="BD22" s="55" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="BE22" s="55"/>
       <c r="BF22" s="55"/>
@@ -6382,7 +6402,7 @@
       </c>
       <c r="BK22" s="54"/>
       <c r="BL22" s="58" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="BM22" s="58"/>
       <c r="BN22" s="58"/>
@@ -6398,12 +6418,12 @@
     <row r="23" customFormat="false" ht="180" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="43"/>
       <c r="B23" s="57" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C23" s="57"/>
       <c r="D23" s="57"/>
       <c r="E23" s="53" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F23" s="53"/>
       <c r="G23" s="53"/>
@@ -6425,7 +6445,7 @@
       <c r="W23" s="53"/>
       <c r="X23" s="53"/>
       <c r="Y23" s="53" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="Z23" s="53"/>
       <c r="AA23" s="53"/>
@@ -6451,24 +6471,28 @@
       <c r="AU23" s="53"/>
       <c r="AV23" s="53"/>
       <c r="AW23" s="53"/>
-      <c r="AX23" s="54"/>
+      <c r="AX23" s="54" t="s">
+        <v>64</v>
+      </c>
       <c r="AY23" s="54"/>
       <c r="AZ23" s="54"/>
       <c r="BA23" s="54"/>
       <c r="BB23" s="54"/>
       <c r="BC23" s="54"/>
-      <c r="BD23" s="55"/>
+      <c r="BD23" s="55" t="s">
+        <v>65</v>
+      </c>
       <c r="BE23" s="55"/>
       <c r="BF23" s="55"/>
       <c r="BG23" s="55"/>
       <c r="BH23" s="55"/>
       <c r="BI23" s="55"/>
       <c r="BJ23" s="54" t="s">
-        <v>64</v>
+        <v>46</v>
       </c>
       <c r="BK23" s="54"/>
       <c r="BL23" s="58" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="BM23" s="58"/>
       <c r="BN23" s="58"/>
@@ -7847,7 +7871,7 @@
     <row r="4" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="44"/>
       <c r="B4" s="60" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C4" s="60"/>
       <c r="D4" s="60"/>
@@ -7859,7 +7883,7 @@
       <c r="J4" s="60"/>
       <c r="K4" s="60"/>
       <c r="L4" s="60" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="M4" s="60"/>
       <c r="N4" s="60"/>
@@ -7890,7 +7914,7 @@
       <c r="AM4" s="60"/>
       <c r="AN4" s="60"/>
       <c r="AO4" s="60" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="AP4" s="60"/>
       <c r="AQ4" s="60"/>
@@ -7901,7 +7925,7 @@
       <c r="AV4" s="60"/>
       <c r="AW4" s="60"/>
       <c r="AX4" s="60" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="AY4" s="60"/>
       <c r="AZ4" s="60"/>
@@ -7910,7 +7934,7 @@
       <c r="BC4" s="60"/>
       <c r="BD4" s="60"/>
       <c r="BE4" s="60" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="BF4" s="60"/>
       <c r="BG4" s="60"/>
@@ -7919,7 +7943,7 @@
       <c r="BJ4" s="60"/>
       <c r="BK4" s="60"/>
       <c r="BL4" s="60" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="BM4" s="60"/>
       <c r="BN4" s="60"/>
@@ -8147,7 +8171,7 @@
     <row r="8" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="43"/>
       <c r="B8" s="64" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C8" s="64"/>
       <c r="D8" s="64"/>
@@ -8159,7 +8183,7 @@
       <c r="J8" s="64"/>
       <c r="K8" s="64"/>
       <c r="L8" s="65" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="M8" s="65"/>
       <c r="N8" s="65"/>
@@ -8210,7 +8234,7 @@
       <c r="BC8" s="66"/>
       <c r="BD8" s="66"/>
       <c r="BE8" s="66" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="BF8" s="66"/>
       <c r="BG8" s="66"/>
@@ -8219,7 +8243,7 @@
       <c r="BJ8" s="66"/>
       <c r="BK8" s="66"/>
       <c r="BL8" s="65" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="BM8" s="65"/>
       <c r="BN8" s="65"/>
@@ -8231,7 +8255,7 @@
     <row r="9" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="43"/>
       <c r="B9" s="65" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C9" s="65"/>
       <c r="D9" s="65"/>
@@ -8243,7 +8267,7 @@
       <c r="J9" s="65"/>
       <c r="K9" s="65"/>
       <c r="L9" s="65" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="M9" s="65"/>
       <c r="N9" s="65"/>
@@ -8285,7 +8309,7 @@
       <c r="AV9" s="66"/>
       <c r="AW9" s="66"/>
       <c r="AX9" s="66" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="AY9" s="66"/>
       <c r="AZ9" s="66"/>
@@ -8294,7 +8318,7 @@
       <c r="BC9" s="66"/>
       <c r="BD9" s="66"/>
       <c r="BE9" s="66" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="BF9" s="66"/>
       <c r="BG9" s="66"/>
@@ -8303,7 +8327,7 @@
       <c r="BJ9" s="66"/>
       <c r="BK9" s="66"/>
       <c r="BL9" s="65" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="BM9" s="65"/>
       <c r="BN9" s="65"/>
@@ -8315,7 +8339,7 @@
     <row r="10" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="43"/>
       <c r="B10" s="65" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C10" s="65"/>
       <c r="D10" s="65"/>
@@ -8327,7 +8351,7 @@
       <c r="J10" s="65"/>
       <c r="K10" s="65"/>
       <c r="L10" s="65" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="M10" s="65"/>
       <c r="N10" s="65"/>
@@ -8369,7 +8393,7 @@
       <c r="AV10" s="66"/>
       <c r="AW10" s="66"/>
       <c r="AX10" s="66" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="AY10" s="66"/>
       <c r="AZ10" s="66"/>
@@ -8378,7 +8402,7 @@
       <c r="BC10" s="66"/>
       <c r="BD10" s="66"/>
       <c r="BE10" s="66" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="BF10" s="66"/>
       <c r="BG10" s="66"/>
@@ -8387,7 +8411,7 @@
       <c r="BJ10" s="66"/>
       <c r="BK10" s="66"/>
       <c r="BL10" s="65" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="BM10" s="65"/>
       <c r="BN10" s="65"/>
@@ -8399,7 +8423,7 @@
     <row r="11" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="43"/>
       <c r="B11" s="65" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C11" s="65"/>
       <c r="D11" s="65"/>
@@ -8411,7 +8435,7 @@
       <c r="J11" s="65"/>
       <c r="K11" s="65"/>
       <c r="L11" s="65" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="M11" s="65"/>
       <c r="N11" s="65"/>
@@ -8462,7 +8486,7 @@
       <c r="BC11" s="66"/>
       <c r="BD11" s="66"/>
       <c r="BE11" s="66" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="BF11" s="66"/>
       <c r="BG11" s="66"/>
@@ -8471,7 +8495,7 @@
       <c r="BJ11" s="66"/>
       <c r="BK11" s="66"/>
       <c r="BL11" s="65" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="BM11" s="65"/>
       <c r="BN11" s="65"/>
@@ -8483,7 +8507,7 @@
     <row r="12" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="43"/>
       <c r="B12" s="65" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C12" s="65"/>
       <c r="D12" s="65"/>
@@ -8495,7 +8519,7 @@
       <c r="J12" s="65"/>
       <c r="K12" s="65"/>
       <c r="L12" s="65" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="M12" s="65"/>
       <c r="N12" s="65"/>
@@ -8537,7 +8561,7 @@
       <c r="AV12" s="66"/>
       <c r="AW12" s="66"/>
       <c r="AX12" s="66" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="AY12" s="66"/>
       <c r="AZ12" s="66"/>
@@ -8546,7 +8570,7 @@
       <c r="BC12" s="66"/>
       <c r="BD12" s="66"/>
       <c r="BE12" s="66" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="BF12" s="66"/>
       <c r="BG12" s="66"/>
@@ -8555,7 +8579,7 @@
       <c r="BJ12" s="66"/>
       <c r="BK12" s="66"/>
       <c r="BL12" s="65" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="BM12" s="65"/>
       <c r="BN12" s="65"/>
@@ -8567,7 +8591,7 @@
     <row r="13" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="43"/>
       <c r="B13" s="65" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C13" s="65"/>
       <c r="D13" s="65"/>
@@ -8579,7 +8603,7 @@
       <c r="J13" s="65"/>
       <c r="K13" s="65"/>
       <c r="L13" s="65" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M13" s="65"/>
       <c r="N13" s="65"/>
@@ -8621,7 +8645,7 @@
       <c r="AV13" s="66"/>
       <c r="AW13" s="66"/>
       <c r="AX13" s="66" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="AY13" s="66"/>
       <c r="AZ13" s="66"/>
@@ -8630,7 +8654,7 @@
       <c r="BC13" s="66"/>
       <c r="BD13" s="66"/>
       <c r="BE13" s="66" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="BF13" s="66"/>
       <c r="BG13" s="66"/>
@@ -8639,7 +8663,7 @@
       <c r="BJ13" s="66"/>
       <c r="BK13" s="66"/>
       <c r="BL13" s="65" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="BM13" s="65"/>
       <c r="BN13" s="65"/>
@@ -13301,7 +13325,7 @@
       <c r="J3" s="47"/>
       <c r="K3" s="47"/>
       <c r="L3" s="47" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="M3" s="47"/>
       <c r="N3" s="47"/>
@@ -13661,7 +13685,7 @@
     <row r="8" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="43"/>
       <c r="B8" s="66" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C8" s="66"/>
       <c r="D8" s="66"/>
@@ -13673,7 +13697,7 @@
       <c r="J8" s="66"/>
       <c r="K8" s="66"/>
       <c r="L8" s="65" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="M8" s="65"/>
       <c r="N8" s="65"/>
@@ -13724,7 +13748,7 @@
       <c r="BC8" s="67"/>
       <c r="BD8" s="67"/>
       <c r="BE8" s="66" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="BF8" s="66"/>
       <c r="BG8" s="66"/>
@@ -13733,7 +13757,7 @@
       <c r="BJ8" s="66"/>
       <c r="BK8" s="66"/>
       <c r="BL8" s="65" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="BM8" s="65"/>
       <c r="BN8" s="65"/>
@@ -13745,7 +13769,7 @@
     <row r="9" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="43"/>
       <c r="B9" s="66" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C9" s="66"/>
       <c r="D9" s="66"/>
@@ -13757,7 +13781,7 @@
       <c r="J9" s="66"/>
       <c r="K9" s="66"/>
       <c r="L9" s="65" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="M9" s="65"/>
       <c r="N9" s="65"/>
@@ -13808,7 +13832,7 @@
       <c r="BC9" s="67"/>
       <c r="BD9" s="67"/>
       <c r="BE9" s="66" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="BF9" s="66"/>
       <c r="BG9" s="66"/>
@@ -13817,7 +13841,7 @@
       <c r="BJ9" s="66"/>
       <c r="BK9" s="66"/>
       <c r="BL9" s="65" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="BM9" s="65"/>
       <c r="BN9" s="65"/>
@@ -13829,7 +13853,7 @@
     <row r="10" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="43"/>
       <c r="B10" s="66" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C10" s="66"/>
       <c r="D10" s="66"/>
@@ -13841,7 +13865,7 @@
       <c r="J10" s="66"/>
       <c r="K10" s="66"/>
       <c r="L10" s="65" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="M10" s="65"/>
       <c r="N10" s="65"/>
@@ -13892,7 +13916,7 @@
       <c r="BC10" s="67"/>
       <c r="BD10" s="67"/>
       <c r="BE10" s="66" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="BF10" s="66"/>
       <c r="BG10" s="66"/>
@@ -13901,7 +13925,7 @@
       <c r="BJ10" s="66"/>
       <c r="BK10" s="66"/>
       <c r="BL10" s="65" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="BM10" s="65"/>
       <c r="BN10" s="65"/>
@@ -13913,7 +13937,7 @@
     <row r="11" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="43"/>
       <c r="B11" s="66" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C11" s="66"/>
       <c r="D11" s="66"/>
@@ -13925,7 +13949,7 @@
       <c r="J11" s="66"/>
       <c r="K11" s="66"/>
       <c r="L11" s="65" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="M11" s="65"/>
       <c r="N11" s="65"/>
@@ -13976,7 +14000,7 @@
       <c r="BC11" s="67"/>
       <c r="BD11" s="67"/>
       <c r="BE11" s="66" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="BF11" s="66"/>
       <c r="BG11" s="66"/>
@@ -13985,7 +14009,7 @@
       <c r="BJ11" s="66"/>
       <c r="BK11" s="66"/>
       <c r="BL11" s="65" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="BM11" s="65"/>
       <c r="BN11" s="65"/>
@@ -13997,7 +14021,7 @@
     <row r="12" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="43"/>
       <c r="B12" s="66" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C12" s="66"/>
       <c r="D12" s="66"/>
@@ -14009,7 +14033,7 @@
       <c r="J12" s="66"/>
       <c r="K12" s="66"/>
       <c r="L12" s="65" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="M12" s="65"/>
       <c r="N12" s="65"/>
@@ -14060,7 +14084,7 @@
       <c r="BC12" s="67"/>
       <c r="BD12" s="67"/>
       <c r="BE12" s="66" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="BF12" s="66"/>
       <c r="BG12" s="66"/>
@@ -14069,7 +14093,7 @@
       <c r="BJ12" s="66"/>
       <c r="BK12" s="66"/>
       <c r="BL12" s="65" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="BM12" s="65"/>
       <c r="BN12" s="65"/>

</xml_diff>